<commit_message>
ajuste do modelo conceitual e dicionário, adicionando tabelas e atributos e atualização do código do DBeaver.
</commit_message>
<xml_diff>
--- a/documentos/modelo_dicionario_de_dados.xlsx
+++ b/documentos/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="264">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -81,145 +81,154 @@
     <t xml:space="preserve">id</t>
   </si>
   <si>
+    <t xml:space="preserve">INTEGER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">auto increment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primaria de identificação do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_funcionario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEXT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo nome_funcionario da tabela funcionario.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIQUE(id, id_cargo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cargo.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do cpf do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cadastro do status do funcionario(0,1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_cadastro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(DATETIME ('now', 'localtime'))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do registro do funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">equipamento</t>
+  </si>
+  <si>
     <t xml:space="preserve">INT</t>
   </si>
   <si>
-    <t xml:space="preserve">PK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NÃO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">auto increment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave primaria de identificação do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">text</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo do nome do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_cargo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNIQUE(id, id_cargo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tabela/cargo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo do cpf do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cadastro do status do funcionario(0,1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data_cadastro</t>
+    <t xml:space="preserve">Chave primaria de identificação do equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nenhum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do nome do equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tabela/marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo da marca de origem do equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tabela/modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo referente ao modelo do equipamento utilizado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tabela/tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Série do equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cadastro do status do equipamento(0,1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tabela/cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo destinado ao cliente que usa o equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_funcionario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tabela/funcionário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo referente ao cadastro do equipamento.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">serial_number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIQUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">imei</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SIM</t>
   </si>
   <si>
     <t xml:space="preserve">datetime(‘now’, ‘localtime’)</t>
   </si>
   <si>
-    <t xml:space="preserve">Campo do registro do funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">equipamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave primaria de identificação do equipamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_equipamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEXT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nenhum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo do nome do equipamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_marca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tabela/marca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo da marca de origem do equipamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_modelo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tabela/modelo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo referente ao modelo do equipamento utilizado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_tipo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tabela/tipo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Série do equipamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cadastro do status do equipamento(0,1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tabela/cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo destinado ao cliente que usa o equipamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_funcionario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tabela/funcionário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo referente ao cadastro do equipamento.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">serial_number</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNIQUE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">imei</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIM</t>
-  </si>
-  <si>
     <t xml:space="preserve">cliente</t>
   </si>
   <si>
     <t xml:space="preserve">Chave primaria de identificação do cliente</t>
   </si>
   <si>
-    <t xml:space="preserve">e-mail</t>
+    <t xml:space="preserve">email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo email da tabela cliente.</t>
   </si>
   <si>
     <t xml:space="preserve">nome_cliente</t>
@@ -231,54 +240,57 @@
     <t xml:space="preserve">cadastro do status do cliente(0,1)</t>
   </si>
   <si>
+    <t xml:space="preserve">funcionario.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo de cadastro do cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_funcionario_cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tabela/equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipamento que se encontra em posse do cliente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primaria de identificação do cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome do cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">situacao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primaria de identificação da situacao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_situacao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Situação atual dos dados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primaria de identificação da marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_marca</t>
+  </si>
+  <si>
     <t xml:space="preserve">tabela/funionario</t>
   </si>
   <si>
-    <t xml:space="preserve">Campo de cadastro do cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_funcionario_cargo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tabela/equipamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equipamento que se encontra em posse do cliente.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cargo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave primaria de identificação do cargo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_cargo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome do cargo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">situacao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave primaria de identificação da situacao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_situacao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Situação atual dos dados</t>
-  </si>
-  <si>
-    <t xml:space="preserve">marca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave primaria de identificação da marca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_marca</t>
-  </si>
-  <si>
     <t xml:space="preserve">Chave entrageira de indetificação o funcionário que efetuo o cadastro. Referência composta entre id_funcionario e id_funcionario_cargo.</t>
   </si>
   <si>
@@ -297,6 +309,327 @@
     <t xml:space="preserve">nome_tipo</t>
   </si>
   <si>
+    <t xml:space="preserve">categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária de identificação da tabela categoria.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo nome_categoria da tabela categoria.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave estrangeira que referencia funcionario.id.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">funcionario.id_cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave estrangeira que referencia funcionario.id_cargo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo status da tabela categoria.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo data_cadastro da tabela categoria.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">servico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária de identificação da tabela servico.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_servico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo nome_servico da tabela servico.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categoria.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave estrangeira que referencia categoria.id.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo preco da tabela servico.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">horas_trabalho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo horas_trabalho da tabela servico.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo status da tabela servico.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo data_cadastro da tabela servico.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária de identificação da tabela peca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_peca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo nome_peca da tabela peca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preco_de_compra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo preco_de_compra da tabela peca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preco_venda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo preco_venda da tabela peca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">estoque_real</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo estoque_real da tabela peca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo status da tabela peca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo data_cadastro da tabela peca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ordem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária de identificação da ordem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cliente.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cliente relacionado à ordem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_funcionario_abertura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funcionário responsável pela abertura da ordem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo do funcionário responsável pela abertura; CHECK (id_funcionario_cargo = 1 OR id_funcionario_cargo = 2).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_situacao_atual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Situação atual da ordem de serviço.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_abertura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(DATETIME('now','localtime'))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data e hora de abertura da ordem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_fechamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data e hora de fechamento da ordem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">descricao_defeito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descrição do defeito informado pelo cliente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">defeito_constatado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descrição do defeito constatado pelo técnico.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valor_total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor total da ordem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_forma_pagamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">forma_pagamento.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forma de pagamento associada à ordem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_tecnico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Técnico responsável pela execução da ordem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_tecnico_cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo do técnico; CHECK (id_tecnico_cargo = 3).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ordem_situacao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária do histórico de situação.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_ordem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ordem.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordem relacionada ao histórico de situação.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_situacao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">situacao_os.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Situação atribuída à ordem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Técnico responsável pela alteração da situação.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_situacao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data e hora em que a situação foi registrada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">forma_pagamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária da forma de pagamento.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_forma_pagamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome da forma de pagamento; COLLATE NOCASE UNIQUE.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funcionário responsável pelo cadastro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo do funcionário responsável pelo cadastro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data e hora do cadastro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status do cadastro da forma de pagamento.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">situacao_os</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária da situação da ordem de serviço.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome da situação; COLLATE NOCASE UNIQUE.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status da situação.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ordem_peca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordem à qual a peça foi associada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_peca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peca.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peça utilizada na ordem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quantidade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantidade de peças utilizadas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valor_unitario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor unitário da peça no momento da utilização.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Técnico responsável pelo uso da peça.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data e hora do registro da peça na ordem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ordem_servico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primária do item de serviço.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_servico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">servico.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serviço executado na ordem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordem na qual o serviço foi executado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_execucao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data e hora da execução do serviço.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quantidade_servico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantidade de vezes que o serviço foi executado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Técnico responsável pela execução.</t>
+  </si>
+  <si>
     <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
   </si>
   <si>
@@ -412,9 +745,6 @@
   </si>
   <si>
     <t xml:space="preserve">Data de nascimento para cálculo de idade.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">email</t>
   </si>
   <si>
     <t xml:space="preserve">NULL</t>
@@ -493,7 +823,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -581,6 +911,13 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="13"/>
       <color rgb="FF1E3A8A"/>
@@ -589,7 +926,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -611,7 +948,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF972F"/>
-        <bgColor rgb="FFFFCC00"/>
+        <bgColor rgb="FFFF7A00"/>
       </patternFill>
     </fill>
     <fill>
@@ -623,7 +960,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF3838"/>
-        <bgColor rgb="FFFF0000"/>
+        <bgColor rgb="FFCC3366"/>
       </patternFill>
     </fill>
     <fill>
@@ -647,13 +984,67 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF6A00FF"/>
-        <bgColor rgb="FF800080"/>
+        <bgColor rgb="FF8A2BE2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF66B3"/>
         <bgColor rgb="FFFF90F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000099"/>
+        <bgColor rgb="FF000080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00994D"/>
+        <bgColor rgb="FF00A86B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF990000"/>
+        <bgColor rgb="FF800000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF7A00"/>
+        <bgColor rgb="FFFF972F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FF7F"/>
+        <bgColor rgb="FF00FFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00A86B"/>
+        <bgColor rgb="FF00994D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF8A2BE2"/>
+        <bgColor rgb="FF6A00FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCC3366"/>
+        <bgColor rgb="FFFF3838"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4C78A8"/>
+        <bgColor rgb="FF808080"/>
       </patternFill>
     </fill>
   </fills>
@@ -706,7 +1097,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="59">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -731,34 +1122,190 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -767,14 +1314,14 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -785,74 +1332,6 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -868,22 +1347,22 @@
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FFFF3838"/>
+      <rgbColor rgb="FF00FF7F"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF990000"/>
       <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF000099"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF6A00FF"/>
-      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF00994D"/>
       <rgbColor rgb="FFC0C0C0"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF729FCF"/>
-      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFCC3366"/>
       <rgbColor rgb="FFF8FAFC"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
@@ -911,17 +1390,17 @@
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF972F"/>
-      <rgbColor rgb="FFFF3838"/>
-      <rgbColor rgb="FF475569"/>
+      <rgbColor rgb="FFFF7A00"/>
+      <rgbColor rgb="FF4C78A8"/>
       <rgbColor rgb="FF77BC65"/>
       <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF00A86B"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF8A2BE2"/>
       <rgbColor rgb="FF1E3A8A"/>
-      <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="FF475569"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -1107,7 +1586,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J121"/>
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
@@ -1233,7 +1712,6 @@
       <c r="I11" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="J11" s="8"/>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
@@ -1278,12 +1756,12 @@
       <c r="F13" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="G13" s="9" t="n">
-        <v>1</v>
+      <c r="G13" s="9" t="s">
+        <v>33</v>
       </c>
       <c r="H13" s="9"/>
       <c r="I13" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J13" s="10"/>
     </row>
@@ -1292,7 +1770,7 @@
         <v>17</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>25</v>
@@ -1303,23 +1781,23 @@
         <v>21</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H14" s="8"/>
       <c r="I14" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J14" s="8"/>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>18</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D15" s="14"/>
       <c r="E15" s="14" t="s">
@@ -1333,22 +1811,22 @@
       </c>
       <c r="H15" s="15"/>
       <c r="I15" s="16" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="D16" s="18"/>
       <c r="E16" s="18" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F16" s="18" t="s">
         <v>21</v>
@@ -1356,18 +1834,18 @@
       <c r="G16" s="17"/>
       <c r="H16" s="15"/>
       <c r="I16" s="19" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D17" s="14"/>
       <c r="E17" s="14" t="s">
@@ -1378,21 +1856,21 @@
       </c>
       <c r="G17" s="13"/>
       <c r="H17" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I17" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D18" s="18"/>
       <c r="E18" s="18" t="s">
@@ -1403,21 +1881,21 @@
       </c>
       <c r="G18" s="17"/>
       <c r="H18" s="15" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I18" s="19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D19" s="18"/>
       <c r="E19" s="18"/>
@@ -1426,21 +1904,21 @@
       </c>
       <c r="G19" s="17"/>
       <c r="H19" s="15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I19" s="19" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D20" s="18"/>
       <c r="E20" s="18"/>
@@ -1450,18 +1928,18 @@
       <c r="G20" s="17"/>
       <c r="H20" s="17"/>
       <c r="I20" s="20" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D21" s="18"/>
       <c r="E21" s="18" t="s">
@@ -1472,21 +1950,21 @@
       </c>
       <c r="G21" s="17"/>
       <c r="H21" s="17" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I21" s="19" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D22" s="18"/>
       <c r="E22" s="18" t="s">
@@ -1497,21 +1975,21 @@
       </c>
       <c r="G22" s="17"/>
       <c r="H22" s="17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I22" s="19" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D23" s="18"/>
       <c r="E23" s="18" t="s">
@@ -1521,47 +1999,47 @@
         <v>21</v>
       </c>
       <c r="G23" s="17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H23" s="17"/>
       <c r="I23" s="19" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D24" s="18"/>
       <c r="E24" s="18" t="s">
         <v>28</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G24" s="17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H24" s="17"/>
       <c r="I24" s="19" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="D25" s="18"/>
       <c r="E25" s="18" t="s">
@@ -1571,16 +2049,16 @@
         <v>21</v>
       </c>
       <c r="G25" s="17" t="s">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="H25" s="17"/>
       <c r="I25" s="19" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="21" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B26" s="10" t="s">
         <v>18</v>
@@ -1600,37 +2078,39 @@
       </c>
       <c r="H26" s="10"/>
       <c r="I26" s="22" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="B27" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="C27" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="G27" s="24"/>
-      <c r="H27" s="24"/>
-      <c r="I27" s="24"/>
+      <c r="B27" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G27" s="9"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="D28" s="14"/>
       <c r="E28" s="14"/>
@@ -1640,12 +2120,12 @@
       <c r="G28" s="13"/>
       <c r="H28" s="10"/>
       <c r="I28" s="16" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B29" s="10" t="s">
         <v>32</v>
@@ -1658,18 +2138,20 @@
       <c r="F29" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G29" s="13"/>
+      <c r="G29" s="13" t="s">
+        <v>33</v>
+      </c>
       <c r="H29" s="13"/>
       <c r="I29" s="22" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="21" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C30" s="17" t="s">
         <v>19</v>
@@ -1683,21 +2165,21 @@
       </c>
       <c r="G30" s="17"/>
       <c r="H30" s="17" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I30" s="19" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D31" s="18"/>
       <c r="E31" s="18" t="s">
@@ -1708,34 +2190,36 @@
       </c>
       <c r="G31" s="17"/>
       <c r="H31" s="17" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I31" s="19" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="B32" s="24" t="s">
-        <v>34</v>
-      </c>
-      <c r="C32" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="G32" s="24"/>
-      <c r="H32" s="24"/>
-      <c r="I32" s="24"/>
+      <c r="A32" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="B32" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="C32" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="D32" s="25"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="G32" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="H32" s="25"/>
+      <c r="I32" s="25"/>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="25" t="s">
-        <v>74</v>
+      <c r="A33" s="26" t="s">
+        <v>77</v>
       </c>
       <c r="B33" s="10" t="s">
         <v>18</v>
@@ -1755,18 +2239,18 @@
       </c>
       <c r="H33" s="10"/>
       <c r="I33" s="22" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="25" t="s">
-        <v>74</v>
+      <c r="A34" s="26" t="s">
+        <v>77</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="D34" s="14"/>
       <c r="E34" s="14"/>
@@ -1774,16 +2258,16 @@
         <v>21</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H34" s="10"/>
       <c r="I34" s="16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="26" t="s">
         <v>77</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="25" t="s">
-        <v>74</v>
       </c>
       <c r="B35" s="15" t="s">
         <v>32</v>
@@ -1796,23 +2280,23 @@
       <c r="F35" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="G35" s="17" t="n">
-        <v>1</v>
+      <c r="G35" s="17" t="s">
+        <v>33</v>
       </c>
       <c r="H35" s="17"/>
       <c r="I35" s="20" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="26" t="s">
-        <v>78</v>
+      <c r="A36" s="27" t="s">
+        <v>81</v>
       </c>
       <c r="B36" s="15" t="s">
         <v>18</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D36" s="18"/>
       <c r="E36" s="18" t="s">
@@ -1826,18 +2310,18 @@
       </c>
       <c r="H36" s="15"/>
       <c r="I36" s="20" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="26" t="s">
-        <v>78</v>
+      <c r="A37" s="27" t="s">
+        <v>81</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="D37" s="14"/>
       <c r="E37" s="14"/>
@@ -1845,43 +2329,43 @@
         <v>21</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H37" s="10"/>
       <c r="I37" s="16" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="27" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="26" t="s">
-        <v>78</v>
-      </c>
       <c r="B38" s="15" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C38" s="17" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="D38" s="18"/>
       <c r="E38" s="18"/>
       <c r="F38" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="G38" s="27" t="s">
-        <v>35</v>
+      <c r="G38" s="28" t="s">
+        <v>64</v>
       </c>
       <c r="H38" s="15"/>
       <c r="I38" s="19"/>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="26" t="s">
-        <v>78</v>
+      <c r="A39" s="27" t="s">
+        <v>81</v>
       </c>
       <c r="B39" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D39" s="14"/>
       <c r="E39" s="14"/>
@@ -1893,18 +2377,18 @@
       </c>
       <c r="H39" s="10"/>
       <c r="I39" s="22" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="28" t="s">
-        <v>82</v>
+      <c r="A40" s="29" t="s">
+        <v>85</v>
       </c>
       <c r="B40" s="10" t="s">
         <v>18</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D40" s="14"/>
       <c r="E40" s="14" t="s">
@@ -1918,18 +2402,18 @@
       </c>
       <c r="H40" s="10"/>
       <c r="I40" s="22" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="28" t="s">
-        <v>82</v>
+      <c r="A41" s="29" t="s">
+        <v>85</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="D41" s="14"/>
       <c r="E41" s="14"/>
@@ -1937,22 +2421,22 @@
         <v>21</v>
       </c>
       <c r="G41" s="13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H41" s="10"/>
       <c r="I41" s="16" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="28" t="s">
-        <v>82</v>
+      <c r="A42" s="29" t="s">
+        <v>85</v>
       </c>
       <c r="B42" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C42" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D42" s="18"/>
       <c r="E42" s="18"/>
@@ -1964,18 +2448,18 @@
       </c>
       <c r="H42" s="17"/>
       <c r="I42" s="20" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="29" t="s">
-        <v>82</v>
+      <c r="A43" s="30" t="s">
+        <v>85</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C43" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D43" s="18"/>
       <c r="E43" s="18" t="s">
@@ -1986,21 +2470,21 @@
       </c>
       <c r="G43" s="17"/>
       <c r="H43" s="17" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="I43" s="19" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="30" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="29" t="s">
-        <v>82</v>
-      </c>
       <c r="B44" s="15" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C44" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D44" s="18"/>
       <c r="E44" s="18" t="s">
@@ -2011,21 +2495,21 @@
       </c>
       <c r="G44" s="17"/>
       <c r="H44" s="17" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I44" s="19" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="30" t="s">
-        <v>87</v>
+      <c r="A45" s="31" t="s">
+        <v>91</v>
       </c>
       <c r="B45" s="10" t="s">
         <v>18</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D45" s="14"/>
       <c r="E45" s="14" t="s">
@@ -2039,18 +2523,18 @@
       </c>
       <c r="H45" s="10"/>
       <c r="I45" s="22" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="30" t="s">
-        <v>87</v>
+      <c r="A46" s="31" t="s">
+        <v>91</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="D46" s="14"/>
       <c r="E46" s="14"/>
@@ -2058,22 +2542,22 @@
         <v>21</v>
       </c>
       <c r="G46" s="13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H46" s="10"/>
       <c r="I46" s="16" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="30" t="s">
-        <v>87</v>
+      <c r="A47" s="31" t="s">
+        <v>91</v>
       </c>
       <c r="B47" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C47" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D47" s="18"/>
       <c r="E47" s="18"/>
@@ -2085,18 +2569,18 @@
       </c>
       <c r="H47" s="17"/>
       <c r="I47" s="20" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="31" t="s">
-        <v>87</v>
+      <c r="A48" s="32" t="s">
+        <v>91</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C48" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D48" s="18"/>
       <c r="E48" s="18" t="s">
@@ -2107,21 +2591,21 @@
       </c>
       <c r="G48" s="17"/>
       <c r="H48" s="17" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="I48" s="19" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="31" t="s">
-        <v>87</v>
+      <c r="A49" s="32" t="s">
+        <v>91</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C49" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D49" s="18"/>
       <c r="E49" s="18" t="s">
@@ -2132,21 +2616,21 @@
       </c>
       <c r="G49" s="17"/>
       <c r="H49" s="17" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I49" s="19" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="32" t="s">
-        <v>89</v>
+      <c r="A50" s="33" t="s">
+        <v>93</v>
       </c>
       <c r="B50" s="10" t="s">
         <v>18</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D50" s="14"/>
       <c r="E50" s="14" t="s">
@@ -2160,18 +2644,18 @@
       </c>
       <c r="H50" s="10"/>
       <c r="I50" s="22" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="32" t="s">
-        <v>89</v>
+      <c r="A51" s="33" t="s">
+        <v>93</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C51" s="13" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="D51" s="14"/>
       <c r="E51" s="14"/>
@@ -2179,22 +2663,22 @@
         <v>21</v>
       </c>
       <c r="G51" s="13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H51" s="10"/>
       <c r="I51" s="16" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="32" t="s">
-        <v>89</v>
+      <c r="A52" s="33" t="s">
+        <v>93</v>
       </c>
       <c r="B52" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C52" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D52" s="18"/>
       <c r="E52" s="18"/>
@@ -2206,18 +2690,18 @@
       </c>
       <c r="H52" s="17"/>
       <c r="I52" s="20" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="33" t="s">
-        <v>89</v>
+      <c r="A53" s="34" t="s">
+        <v>93</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C53" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D53" s="18"/>
       <c r="E53" s="18" t="s">
@@ -2228,21 +2712,21 @@
       </c>
       <c r="G53" s="17"/>
       <c r="H53" s="17" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="I53" s="19" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="33" t="s">
-        <v>89</v>
+      <c r="A54" s="34" t="s">
+        <v>93</v>
       </c>
       <c r="B54" s="15" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C54" s="17" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D54" s="18"/>
       <c r="E54" s="18" t="s">
@@ -2253,78 +2737,1598 @@
       </c>
       <c r="G54" s="17"/>
       <c r="H54" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="I54" s="19" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="B55" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C55" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F55" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G55" s="9"/>
+      <c r="H55" s="8"/>
+      <c r="I55" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D56" s="9"/>
+      <c r="E56" s="9"/>
+      <c r="F56" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G56" s="9"/>
+      <c r="H56" s="8"/>
+      <c r="I56" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="B57" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D57" s="9"/>
+      <c r="E57" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F57" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G57" s="9"/>
+      <c r="H57" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="I54" s="19" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="10"/>
-      <c r="B55" s="10"/>
-      <c r="C55" s="13"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="14"/>
-      <c r="F55" s="14"/>
-      <c r="G55" s="13"/>
-      <c r="H55" s="10"/>
-      <c r="I55" s="16"/>
-    </row>
-    <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="15"/>
-      <c r="B56" s="15"/>
-      <c r="C56" s="17"/>
-      <c r="D56" s="18"/>
-      <c r="E56" s="18"/>
-      <c r="F56" s="18"/>
-      <c r="G56" s="17"/>
-      <c r="H56" s="15"/>
-      <c r="I56" s="19"/>
-    </row>
-    <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="10"/>
-      <c r="B57" s="10"/>
-      <c r="C57" s="13"/>
-      <c r="D57" s="14"/>
-      <c r="E57" s="14"/>
-      <c r="F57" s="14"/>
-      <c r="G57" s="13"/>
-      <c r="H57" s="10"/>
-      <c r="I57" s="16"/>
+      <c r="I57" s="8" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="15"/>
-      <c r="B58" s="15"/>
-      <c r="C58" s="17"/>
-      <c r="D58" s="18"/>
-      <c r="E58" s="18"/>
-      <c r="F58" s="18"/>
-      <c r="G58" s="17"/>
-      <c r="H58" s="15"/>
-      <c r="I58" s="19"/>
+      <c r="A58" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D58" s="9"/>
+      <c r="E58" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F58" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G58" s="9"/>
+      <c r="H58" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="I58" s="8" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="10"/>
-      <c r="B59" s="10"/>
-      <c r="C59" s="13"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="14"/>
-      <c r="F59" s="14"/>
-      <c r="G59" s="13"/>
-      <c r="H59" s="10"/>
-      <c r="I59" s="16"/>
+      <c r="A59" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="B59" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D59" s="9"/>
+      <c r="E59" s="9"/>
+      <c r="F59" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G59" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H59" s="8"/>
+      <c r="I59" s="8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D60" s="9"/>
+      <c r="E60" s="9"/>
+      <c r="F60" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G60" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="H60" s="8"/>
+      <c r="I60" s="8" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="B61" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C61" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D61" s="9"/>
+      <c r="E61" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F61" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G61" s="9"/>
+      <c r="H61" s="8"/>
+      <c r="I61" s="8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C62" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D62" s="9"/>
+      <c r="E62" s="9"/>
+      <c r="F62" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G62" s="9"/>
+      <c r="H62" s="8"/>
+      <c r="I62" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="B63" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C63" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D63" s="9"/>
+      <c r="E63" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F63" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G63" s="9"/>
+      <c r="H63" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="I63" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C64" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D64" s="9"/>
+      <c r="E64" s="9"/>
+      <c r="F64" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G64" s="9"/>
+      <c r="H64" s="8"/>
+      <c r="I64" s="8" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="B65" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C65" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="D65" s="9"/>
+      <c r="E65" s="9"/>
+      <c r="F65" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G65" s="9"/>
+      <c r="H65" s="8"/>
+      <c r="I65" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C66" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D66" s="9"/>
+      <c r="E66" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F66" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G66" s="9"/>
+      <c r="H66" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="I66" s="8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C67" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D67" s="9"/>
+      <c r="E67" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F67" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G67" s="9"/>
+      <c r="H67" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="I67" s="8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C68" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D68" s="9"/>
+      <c r="E68" s="9"/>
+      <c r="F68" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G68" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H68" s="8"/>
+      <c r="I68" s="8" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="B69" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C69" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D69" s="9"/>
+      <c r="E69" s="9"/>
+      <c r="F69" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G69" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="H69" s="8"/>
+      <c r="I69" s="8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C70" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D70" s="9"/>
+      <c r="E70" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F70" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G70" s="9"/>
+      <c r="H70" s="8"/>
+      <c r="I70" s="8" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="B71" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C71" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D71" s="9"/>
+      <c r="E71" s="9"/>
+      <c r="F71" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G71" s="9"/>
+      <c r="H71" s="8"/>
+      <c r="I71" s="8" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C72" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D72" s="9"/>
+      <c r="E72" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F72" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G72" s="9"/>
+      <c r="H72" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="I72" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="B73" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="C73" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D73" s="9"/>
+      <c r="E73" s="9"/>
+      <c r="F73" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G73" s="9"/>
+      <c r="H73" s="8"/>
+      <c r="I73" s="8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="C74" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D74" s="9"/>
+      <c r="E74" s="9"/>
+      <c r="F74" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G74" s="9"/>
+      <c r="H74" s="8"/>
+      <c r="I74" s="8" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="B75" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C75" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D75" s="9"/>
+      <c r="E75" s="9"/>
+      <c r="F75" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G75" s="9"/>
+      <c r="H75" s="8"/>
+      <c r="I75" s="8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C76" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D76" s="9"/>
+      <c r="E76" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F76" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G76" s="9"/>
+      <c r="H76" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="I76" s="8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="B77" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C77" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D77" s="9"/>
+      <c r="E77" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F77" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G77" s="9"/>
+      <c r="H77" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="I77" s="8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C78" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D78" s="9"/>
+      <c r="E78" s="9"/>
+      <c r="F78" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G78" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H78" s="8"/>
+      <c r="I78" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="B79" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C79" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D79" s="9"/>
+      <c r="E79" s="9"/>
+      <c r="F79" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G79" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="H79" s="8"/>
+      <c r="I79" s="8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C80" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D80" s="39"/>
+      <c r="E80" s="39" t="s">
+        <v>20</v>
+      </c>
+      <c r="F80" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G80" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="H80" s="40"/>
+      <c r="I80" s="41" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="B81" s="41" t="s">
+        <v>54</v>
+      </c>
+      <c r="C81" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D81" s="39"/>
+      <c r="E81" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F81" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G81" s="39"/>
+      <c r="H81" s="40" t="s">
+        <v>132</v>
+      </c>
+      <c r="I81" s="41" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="B82" s="41" t="s">
+        <v>134</v>
+      </c>
+      <c r="C82" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D82" s="39"/>
+      <c r="E82" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F82" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G82" s="39"/>
+      <c r="H82" s="40" t="s">
+        <v>72</v>
+      </c>
+      <c r="I82" s="41" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="B83" s="41" t="s">
+        <v>74</v>
+      </c>
+      <c r="C83" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D83" s="39"/>
+      <c r="E83" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F83" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G83" s="39"/>
+      <c r="H83" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="I83" s="41" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="B84" s="41" t="s">
+        <v>137</v>
+      </c>
+      <c r="C84" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="D84" s="39"/>
+      <c r="E84" s="39"/>
+      <c r="F84" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G84" s="39"/>
+      <c r="H84" s="40"/>
+      <c r="I84" s="41" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="B85" s="41" t="s">
+        <v>139</v>
+      </c>
+      <c r="C85" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="D85" s="39"/>
+      <c r="E85" s="39"/>
+      <c r="F85" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G85" s="39" t="s">
+        <v>140</v>
+      </c>
+      <c r="H85" s="40"/>
+      <c r="I85" s="41" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="B86" s="41" t="s">
+        <v>142</v>
+      </c>
+      <c r="C86" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="D86" s="39"/>
+      <c r="E86" s="39"/>
+      <c r="F86" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G86" s="39" t="s">
+        <v>140</v>
+      </c>
+      <c r="H86" s="40"/>
+      <c r="I86" s="41" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="B87" s="41" t="s">
+        <v>144</v>
+      </c>
+      <c r="C87" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="D87" s="39"/>
+      <c r="E87" s="39"/>
+      <c r="F87" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G87" s="39"/>
+      <c r="H87" s="40"/>
+      <c r="I87" s="41" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="B88" s="41" t="s">
+        <v>146</v>
+      </c>
+      <c r="C88" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="D88" s="39"/>
+      <c r="E88" s="39"/>
+      <c r="F88" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G88" s="39"/>
+      <c r="H88" s="40"/>
+      <c r="I88" s="41" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="B89" s="41" t="s">
+        <v>148</v>
+      </c>
+      <c r="C89" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D89" s="39"/>
+      <c r="E89" s="39"/>
+      <c r="F89" s="39"/>
+      <c r="G89" s="39"/>
+      <c r="H89" s="40"/>
+      <c r="I89" s="41" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="B90" s="41" t="s">
+        <v>150</v>
+      </c>
+      <c r="C90" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D90" s="39"/>
+      <c r="E90" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F90" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G90" s="39"/>
+      <c r="H90" s="40" t="s">
+        <v>151</v>
+      </c>
+      <c r="I90" s="41" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="B91" s="41" t="s">
+        <v>153</v>
+      </c>
+      <c r="C91" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D91" s="39"/>
+      <c r="E91" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F91" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G91" s="39"/>
+      <c r="H91" s="40" t="s">
+        <v>72</v>
+      </c>
+      <c r="I91" s="41" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="B92" s="41" t="s">
+        <v>155</v>
+      </c>
+      <c r="C92" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D92" s="39"/>
+      <c r="E92" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F92" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G92" s="39"/>
+      <c r="H92" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="I92" s="41" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="42" t="s">
+        <v>157</v>
+      </c>
+      <c r="B93" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="C93" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D93" s="39"/>
+      <c r="E93" s="39" t="s">
+        <v>20</v>
+      </c>
+      <c r="F93" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G93" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="H93" s="40"/>
+      <c r="I93" s="41" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="42" t="s">
+        <v>157</v>
+      </c>
+      <c r="B94" s="41" t="s">
+        <v>159</v>
+      </c>
+      <c r="C94" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D94" s="39"/>
+      <c r="E94" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F94" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G94" s="39"/>
+      <c r="H94" s="40" t="s">
+        <v>160</v>
+      </c>
+      <c r="I94" s="41" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="42" t="s">
+        <v>157</v>
+      </c>
+      <c r="B95" s="41" t="s">
+        <v>162</v>
+      </c>
+      <c r="C95" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D95" s="39"/>
+      <c r="E95" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F95" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G95" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="H95" s="40" t="s">
+        <v>163</v>
+      </c>
+      <c r="I95" s="41" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="42" t="s">
+        <v>157</v>
+      </c>
+      <c r="B96" s="41" t="s">
+        <v>153</v>
+      </c>
+      <c r="C96" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D96" s="39"/>
+      <c r="E96" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F96" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G96" s="39"/>
+      <c r="H96" s="40" t="s">
+        <v>72</v>
+      </c>
+      <c r="I96" s="41" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="42" t="s">
+        <v>157</v>
+      </c>
+      <c r="B97" s="41" t="s">
+        <v>155</v>
+      </c>
+      <c r="C97" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D97" s="39"/>
+      <c r="E97" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F97" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G97" s="39"/>
+      <c r="H97" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="I97" s="41" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="42" t="s">
+        <v>157</v>
+      </c>
+      <c r="B98" s="41" t="s">
+        <v>166</v>
+      </c>
+      <c r="C98" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="D98" s="39"/>
+      <c r="E98" s="39"/>
+      <c r="F98" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G98" s="39" t="s">
+        <v>140</v>
+      </c>
+      <c r="H98" s="40"/>
+      <c r="I98" s="41" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="43" t="s">
+        <v>168</v>
+      </c>
+      <c r="B99" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="C99" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D99" s="39"/>
+      <c r="E99" s="39" t="s">
+        <v>20</v>
+      </c>
+      <c r="F99" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G99" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="H99" s="40"/>
+      <c r="I99" s="41" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="43" t="s">
+        <v>168</v>
+      </c>
+      <c r="B100" s="41" t="s">
+        <v>170</v>
+      </c>
+      <c r="C100" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="D100" s="39"/>
+      <c r="E100" s="39"/>
+      <c r="F100" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G100" s="39"/>
+      <c r="H100" s="40"/>
+      <c r="I100" s="41" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="43" t="s">
+        <v>168</v>
+      </c>
+      <c r="B101" s="41" t="s">
+        <v>57</v>
+      </c>
+      <c r="C101" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D101" s="39"/>
+      <c r="E101" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F101" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G101" s="39"/>
+      <c r="H101" s="40" t="s">
+        <v>72</v>
+      </c>
+      <c r="I101" s="41" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="43" t="s">
+        <v>168</v>
+      </c>
+      <c r="B102" s="41" t="s">
+        <v>74</v>
+      </c>
+      <c r="C102" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D102" s="39"/>
+      <c r="E102" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F102" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G102" s="39"/>
+      <c r="H102" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="I102" s="41" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="43" t="s">
+        <v>168</v>
+      </c>
+      <c r="B103" s="41" t="s">
+        <v>35</v>
+      </c>
+      <c r="C103" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="D103" s="39"/>
+      <c r="E103" s="39"/>
+      <c r="F103" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G103" s="39" t="s">
+        <v>140</v>
+      </c>
+      <c r="H103" s="40"/>
+      <c r="I103" s="41" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="43" t="s">
+        <v>168</v>
+      </c>
+      <c r="B104" s="41" t="s">
+        <v>32</v>
+      </c>
+      <c r="C104" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D104" s="39"/>
+      <c r="E104" s="39"/>
+      <c r="F104" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G104" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="H104" s="40"/>
+      <c r="I104" s="41" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="44" t="s">
+        <v>176</v>
+      </c>
+      <c r="B105" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="C105" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D105" s="39"/>
+      <c r="E105" s="39" t="s">
+        <v>20</v>
+      </c>
+      <c r="F105" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G105" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="H105" s="40"/>
+      <c r="I105" s="41" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="44" t="s">
+        <v>176</v>
+      </c>
+      <c r="B106" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="C106" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="D106" s="39"/>
+      <c r="E106" s="39"/>
+      <c r="F106" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G106" s="39"/>
+      <c r="H106" s="40"/>
+      <c r="I106" s="41" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="44" t="s">
+        <v>176</v>
+      </c>
+      <c r="B107" s="41" t="s">
+        <v>32</v>
+      </c>
+      <c r="C107" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D107" s="39"/>
+      <c r="E107" s="39"/>
+      <c r="F107" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G107" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="H107" s="40"/>
+      <c r="I107" s="41" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="45" t="s">
+        <v>180</v>
+      </c>
+      <c r="B108" s="41" t="s">
+        <v>159</v>
+      </c>
+      <c r="C108" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D108" s="39"/>
+      <c r="E108" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F108" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G108" s="39"/>
+      <c r="H108" s="40" t="s">
+        <v>160</v>
+      </c>
+      <c r="I108" s="41" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="45" t="s">
+        <v>180</v>
+      </c>
+      <c r="B109" s="41" t="s">
+        <v>182</v>
+      </c>
+      <c r="C109" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D109" s="39"/>
+      <c r="E109" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F109" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G109" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="H109" s="40" t="s">
+        <v>183</v>
+      </c>
+      <c r="I109" s="41" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="45" t="s">
+        <v>180</v>
+      </c>
+      <c r="B110" s="41" t="s">
+        <v>185</v>
+      </c>
+      <c r="C110" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D110" s="39"/>
+      <c r="E110" s="39"/>
+      <c r="F110" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G110" s="39"/>
+      <c r="H110" s="40"/>
+      <c r="I110" s="41" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="45" t="s">
+        <v>180</v>
+      </c>
+      <c r="B111" s="41" t="s">
+        <v>187</v>
+      </c>
+      <c r="C111" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D111" s="39"/>
+      <c r="E111" s="39"/>
+      <c r="F111" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G111" s="39"/>
+      <c r="H111" s="40"/>
+      <c r="I111" s="41" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="45" t="s">
+        <v>180</v>
+      </c>
+      <c r="B112" s="41" t="s">
+        <v>153</v>
+      </c>
+      <c r="C112" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D112" s="39"/>
+      <c r="E112" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F112" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G112" s="39"/>
+      <c r="H112" s="40" t="s">
+        <v>72</v>
+      </c>
+      <c r="I112" s="41" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="45" t="s">
+        <v>180</v>
+      </c>
+      <c r="B113" s="41" t="s">
+        <v>155</v>
+      </c>
+      <c r="C113" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D113" s="39"/>
+      <c r="E113" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F113" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G113" s="39"/>
+      <c r="H113" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="I113" s="41" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="45" t="s">
+        <v>180</v>
+      </c>
+      <c r="B114" s="41" t="s">
+        <v>166</v>
+      </c>
+      <c r="C114" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="D114" s="39"/>
+      <c r="E114" s="39"/>
+      <c r="F114" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G114" s="39" t="s">
+        <v>140</v>
+      </c>
+      <c r="H114" s="40"/>
+      <c r="I114" s="41" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="46" t="s">
+        <v>191</v>
+      </c>
+      <c r="B115" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="C115" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D115" s="39"/>
+      <c r="E115" s="39" t="s">
+        <v>20</v>
+      </c>
+      <c r="F115" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G115" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="H115" s="40"/>
+      <c r="I115" s="41" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="46" t="s">
+        <v>191</v>
+      </c>
+      <c r="B116" s="41" t="s">
+        <v>193</v>
+      </c>
+      <c r="C116" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D116" s="39"/>
+      <c r="E116" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F116" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G116" s="39"/>
+      <c r="H116" s="40" t="s">
+        <v>194</v>
+      </c>
+      <c r="I116" s="41" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="46" t="s">
+        <v>191</v>
+      </c>
+      <c r="B117" s="41" t="s">
+        <v>159</v>
+      </c>
+      <c r="C117" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D117" s="39"/>
+      <c r="E117" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F117" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G117" s="39"/>
+      <c r="H117" s="40" t="s">
+        <v>160</v>
+      </c>
+      <c r="I117" s="41" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="46" t="s">
+        <v>191</v>
+      </c>
+      <c r="B118" s="41" t="s">
+        <v>197</v>
+      </c>
+      <c r="C118" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="D118" s="39"/>
+      <c r="E118" s="39"/>
+      <c r="F118" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G118" s="39" t="s">
+        <v>140</v>
+      </c>
+      <c r="H118" s="40"/>
+      <c r="I118" s="41" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="46" t="s">
+        <v>191</v>
+      </c>
+      <c r="B119" s="41" t="s">
+        <v>199</v>
+      </c>
+      <c r="C119" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D119" s="39"/>
+      <c r="E119" s="39"/>
+      <c r="F119" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G119" s="39"/>
+      <c r="H119" s="40"/>
+      <c r="I119" s="41" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="46" t="s">
+        <v>191</v>
+      </c>
+      <c r="B120" s="41" t="s">
+        <v>153</v>
+      </c>
+      <c r="C120" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D120" s="39"/>
+      <c r="E120" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F120" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G120" s="39"/>
+      <c r="H120" s="40" t="s">
+        <v>72</v>
+      </c>
+      <c r="I120" s="41" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="46" t="s">
+        <v>191</v>
+      </c>
+      <c r="B121" s="41" t="s">
+        <v>155</v>
+      </c>
+      <c r="C121" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="D121" s="39"/>
+      <c r="E121" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="F121" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G121" s="39"/>
+      <c r="H121" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="I121" s="41" t="s">
+        <v>156</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C15:C26 C28:C31 C33:C59" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C15:C26 C28:C31 C33:C54" type="list">
       <formula1>Validações!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E15:E26 E28:E31 E33:E59" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E15:E26 E28:E31 E33:E54" type="list">
       <formula1>Validações!$B$1:$B$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F15:F26 F28:F31 F33:F59" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F15:F26 F28:F31 F33:F54" type="list">
       <formula1>Validações!$C$1:$C$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2359,361 +4363,361 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>91</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>92</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="B4" s="35" t="s">
-        <v>94</v>
+      <c r="A4" s="47" t="s">
+        <v>204</v>
+      </c>
+      <c r="B4" s="48" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="34" t="s">
-        <v>95</v>
-      </c>
-      <c r="B5" s="35" t="s">
-        <v>96</v>
+      <c r="A5" s="47" t="s">
+        <v>206</v>
+      </c>
+      <c r="B5" s="48" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="34" t="s">
-        <v>97</v>
-      </c>
-      <c r="B6" s="35" t="s">
-        <v>98</v>
+      <c r="A6" s="47" t="s">
+        <v>208</v>
+      </c>
+      <c r="B6" s="48" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="34" t="s">
-        <v>99</v>
-      </c>
-      <c r="B7" s="35" t="s">
-        <v>100</v>
+      <c r="A7" s="47" t="s">
+        <v>210</v>
+      </c>
+      <c r="B7" s="48" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="34" t="s">
-        <v>101</v>
-      </c>
-      <c r="B8" s="35" t="s">
-        <v>102</v>
+      <c r="A8" s="47" t="s">
+        <v>212</v>
+      </c>
+      <c r="B8" s="48" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="34" t="s">
-        <v>103</v>
-      </c>
-      <c r="B9" s="35" t="s">
-        <v>104</v>
+      <c r="A9" s="47" t="s">
+        <v>214</v>
+      </c>
+      <c r="B9" s="48" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="34" t="s">
-        <v>105</v>
-      </c>
-      <c r="B10" s="35" t="s">
-        <v>106</v>
+      <c r="A10" s="47" t="s">
+        <v>216</v>
+      </c>
+      <c r="B10" s="48" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="B11" s="35" t="s">
-        <v>108</v>
+      <c r="A11" s="47" t="s">
+        <v>218</v>
+      </c>
+      <c r="B11" s="48" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="34" t="s">
-        <v>109</v>
-      </c>
-      <c r="B12" s="35" t="s">
-        <v>110</v>
+      <c r="A12" s="47" t="s">
+        <v>220</v>
+      </c>
+      <c r="B12" s="48" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="36" t="s">
-        <v>111</v>
+      <c r="A14" s="49" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="C16" s="6" t="s">
+      <c r="B16" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="C16" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="G16" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="I16" s="6" t="s">
+      <c r="G16" s="50" t="s">
+        <v>224</v>
+      </c>
+      <c r="H16" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="I16" s="50" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D17" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="E17" s="14" t="s">
+      <c r="A17" s="51" t="s">
+        <v>226</v>
+      </c>
+      <c r="B17" s="51" t="s">
+        <v>227</v>
+      </c>
+      <c r="C17" s="52" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="53" t="s">
+        <v>228</v>
+      </c>
+      <c r="E17" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="F17" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="G17" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="I17" s="16" t="s">
-        <v>120</v>
+      <c r="F17" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="52" t="s">
+        <v>229</v>
+      </c>
+      <c r="H17" s="51" t="s">
+        <v>230</v>
+      </c>
+      <c r="I17" s="54" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="B18" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="C18" s="17" t="s">
-        <v>122</v>
-      </c>
-      <c r="D18" s="18" t="s">
-        <v>123</v>
-      </c>
-      <c r="E18" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="F18" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="G18" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="H18" s="15" t="s">
-        <v>124</v>
+      <c r="A18" s="55" t="s">
+        <v>226</v>
+      </c>
+      <c r="B18" s="55" t="s">
+        <v>232</v>
+      </c>
+      <c r="C18" s="56" t="s">
+        <v>233</v>
+      </c>
+      <c r="D18" s="57" t="s">
+        <v>234</v>
+      </c>
+      <c r="E18" s="57" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" s="57" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="56" t="s">
+        <v>230</v>
+      </c>
+      <c r="H18" s="55" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>125</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="D19" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="E19" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="F19" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="G19" s="13" t="s">
-        <v>119</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>126</v>
+      <c r="A19" s="51" t="s">
+        <v>226</v>
+      </c>
+      <c r="B19" s="51" t="s">
+        <v>236</v>
+      </c>
+      <c r="C19" s="52" t="s">
+        <v>233</v>
+      </c>
+      <c r="D19" s="53" t="s">
+        <v>228</v>
+      </c>
+      <c r="E19" s="53" t="s">
+        <v>42</v>
+      </c>
+      <c r="F19" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="G19" s="52" t="s">
+        <v>230</v>
+      </c>
+      <c r="H19" s="51" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="B20" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="C20" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="D20" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="E20" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="G20" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="H20" s="15" t="s">
-        <v>129</v>
+      <c r="A20" s="55" t="s">
+        <v>226</v>
+      </c>
+      <c r="B20" s="55" t="s">
+        <v>238</v>
+      </c>
+      <c r="C20" s="56" t="s">
+        <v>239</v>
+      </c>
+      <c r="D20" s="57" t="s">
+        <v>230</v>
+      </c>
+      <c r="E20" s="57" t="s">
+        <v>42</v>
+      </c>
+      <c r="F20" s="57" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="56" t="s">
+        <v>230</v>
+      </c>
+      <c r="H20" s="55" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="D21" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="E21" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="F21" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="G21" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="H21" s="10" t="s">
-        <v>132</v>
+      <c r="A21" s="51" t="s">
+        <v>226</v>
+      </c>
+      <c r="B21" s="51" t="s">
+        <v>67</v>
+      </c>
+      <c r="C21" s="52" t="s">
+        <v>233</v>
+      </c>
+      <c r="D21" s="53" t="s">
+        <v>234</v>
+      </c>
+      <c r="E21" s="53" t="s">
+        <v>42</v>
+      </c>
+      <c r="F21" s="53" t="s">
+        <v>63</v>
+      </c>
+      <c r="G21" s="52" t="s">
+        <v>241</v>
+      </c>
+      <c r="H21" s="51" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="C22" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="D22" s="18" t="s">
-        <v>117</v>
-      </c>
-      <c r="E22" s="18" t="s">
+      <c r="A22" s="55" t="s">
+        <v>226</v>
+      </c>
+      <c r="B22" s="55" t="s">
+        <v>243</v>
+      </c>
+      <c r="C22" s="56" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" s="57" t="s">
+        <v>228</v>
+      </c>
+      <c r="E22" s="57" t="s">
         <v>28</v>
       </c>
-      <c r="F22" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="G22" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="H22" s="15" t="s">
-        <v>134</v>
-      </c>
-      <c r="I22" s="19" t="s">
-        <v>135</v>
+      <c r="F22" s="57" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" s="56" t="s">
+        <v>230</v>
+      </c>
+      <c r="H22" s="55" t="s">
+        <v>244</v>
+      </c>
+      <c r="I22" s="58" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="E23" s="14" t="s">
+      <c r="A23" s="51" t="s">
+        <v>246</v>
+      </c>
+      <c r="B23" s="51" t="s">
+        <v>243</v>
+      </c>
+      <c r="C23" s="52" t="s">
+        <v>39</v>
+      </c>
+      <c r="D23" s="53" t="s">
+        <v>228</v>
+      </c>
+      <c r="E23" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="F23" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="G23" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="H23" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="I23" s="16" t="s">
-        <v>137</v>
+      <c r="F23" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" s="52" t="s">
+        <v>229</v>
+      </c>
+      <c r="H23" s="51" t="s">
+        <v>230</v>
+      </c>
+      <c r="I23" s="54" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="C24" s="17" t="s">
-        <v>122</v>
-      </c>
-      <c r="D24" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="E24" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="F24" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="G24" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="H24" s="15" t="s">
-        <v>140</v>
+      <c r="A24" s="55" t="s">
+        <v>246</v>
+      </c>
+      <c r="B24" s="55" t="s">
+        <v>248</v>
+      </c>
+      <c r="C24" s="56" t="s">
+        <v>233</v>
+      </c>
+      <c r="D24" s="57" t="s">
+        <v>249</v>
+      </c>
+      <c r="E24" s="57" t="s">
+        <v>42</v>
+      </c>
+      <c r="F24" s="57" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="56" t="s">
+        <v>230</v>
+      </c>
+      <c r="H24" s="55" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D25" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="E25" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="F25" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="G25" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>144</v>
+      <c r="A25" s="51" t="s">
+        <v>246</v>
+      </c>
+      <c r="B25" s="51" t="s">
+        <v>251</v>
+      </c>
+      <c r="C25" s="52" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" s="53" t="s">
+        <v>252</v>
+      </c>
+      <c r="E25" s="53" t="s">
+        <v>42</v>
+      </c>
+      <c r="F25" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="52" t="s">
+        <v>253</v>
+      </c>
+      <c r="H25" s="51" t="s">
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -2737,18 +4741,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>145</v>
+        <v>255</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>28</v>
@@ -2759,53 +4763,53 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>146</v>
+        <v>256</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>147</v>
+        <v>257</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>148</v>
+        <v>258</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>149</v>
+        <v>259</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>150</v>
+        <v>260</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>128</v>
+        <v>239</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>151</v>
+        <v>261</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>152</v>
+        <v>262</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>153</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Criação dos restantes das tábelas do módulo B e Inicio do Módulo C
</commit_message>
<xml_diff>
--- a/documentos/modelo_dicionario_de_dados.xlsx
+++ b/documentos/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="888" uniqueCount="272">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -628,6 +628,30 @@
   </si>
   <si>
     <t xml:space="preserve">Técnico responsável pela execução.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">entrada_peca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peça que será comprada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantidade que foi comprada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preço de compra da peça.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gerente responsável pela compra.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">funcioario.id_cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargo do gerente; CHECK (id_funcionario_cargo = 1).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data e hora da compra da peça.</t>
   </si>
   <si>
     <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
@@ -823,7 +847,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -918,6 +942,12 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="13"/>
       <color rgb="FF1E3A8A"/>
@@ -926,7 +956,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1047,6 +1077,12 @@
         <bgColor rgb="FF808080"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5555FF"/>
+        <bgColor rgb="FF4C78A8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
@@ -1097,7 +1133,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="50">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1122,168 +1158,168 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="17" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -1294,44 +1330,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1385,7 +1385,7 @@
       <rgbColor rgb="FFFF90F3"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF5555FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
@@ -1586,7 +1586,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J121"/>
+  <dimension ref="A1:J128"/>
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
@@ -3325,21 +3325,20 @@
       <c r="B80" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C80" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D80" s="39"/>
-      <c r="E80" s="39" t="s">
+      <c r="C80" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D80" s="9"/>
+      <c r="E80" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F80" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G80" s="39" t="s">
+      <c r="F80" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G80" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H80" s="40"/>
-      <c r="I80" s="41" t="s">
+      <c r="I80" s="8" t="s">
         <v>131</v>
       </c>
     </row>
@@ -3347,24 +3346,24 @@
       <c r="A81" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="B81" s="41" t="s">
+      <c r="B81" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C81" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D81" s="39"/>
-      <c r="E81" s="39" t="s">
+      <c r="C81" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D81" s="9"/>
+      <c r="E81" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F81" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G81" s="39"/>
-      <c r="H81" s="40" t="s">
+      <c r="F81" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G81" s="9"/>
+      <c r="H81" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="I81" s="41" t="s">
+      <c r="I81" s="8" t="s">
         <v>133</v>
       </c>
     </row>
@@ -3372,24 +3371,24 @@
       <c r="A82" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="B82" s="41" t="s">
+      <c r="B82" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="C82" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D82" s="39"/>
-      <c r="E82" s="39" t="s">
+      <c r="C82" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D82" s="9"/>
+      <c r="E82" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F82" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G82" s="39"/>
-      <c r="H82" s="40" t="s">
+      <c r="F82" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G82" s="9"/>
+      <c r="H82" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="I82" s="41" t="s">
+      <c r="I82" s="8" t="s">
         <v>135</v>
       </c>
     </row>
@@ -3397,24 +3396,24 @@
       <c r="A83" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="B83" s="41" t="s">
+      <c r="B83" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C83" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D83" s="39"/>
-      <c r="E83" s="39" t="s">
+      <c r="C83" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D83" s="9"/>
+      <c r="E83" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F83" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G83" s="39"/>
-      <c r="H83" s="40" t="s">
+      <c r="F83" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G83" s="9"/>
+      <c r="H83" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="I83" s="41" t="s">
+      <c r="I83" s="8" t="s">
         <v>136</v>
       </c>
     </row>
@@ -3422,20 +3421,19 @@
       <c r="A84" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="B84" s="41" t="s">
+      <c r="B84" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="C84" s="39" t="s">
+      <c r="C84" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D84" s="39"/>
-      <c r="E84" s="39"/>
-      <c r="F84" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G84" s="39"/>
-      <c r="H84" s="40"/>
-      <c r="I84" s="41" t="s">
+      <c r="D84" s="9"/>
+      <c r="E84" s="9"/>
+      <c r="F84" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G84" s="9"/>
+      <c r="I84" s="8" t="s">
         <v>138</v>
       </c>
     </row>
@@ -3443,22 +3441,21 @@
       <c r="A85" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="B85" s="41" t="s">
+      <c r="B85" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="C85" s="39" t="s">
+      <c r="C85" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D85" s="39"/>
-      <c r="E85" s="39"/>
-      <c r="F85" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G85" s="39" t="s">
+      <c r="D85" s="9"/>
+      <c r="E85" s="9"/>
+      <c r="F85" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G85" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="H85" s="40"/>
-      <c r="I85" s="41" t="s">
+      <c r="I85" s="8" t="s">
         <v>141</v>
       </c>
     </row>
@@ -3466,22 +3463,21 @@
       <c r="A86" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="B86" s="41" t="s">
+      <c r="B86" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="C86" s="39" t="s">
+      <c r="C86" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D86" s="39"/>
-      <c r="E86" s="39"/>
-      <c r="F86" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G86" s="39" t="s">
+      <c r="D86" s="9"/>
+      <c r="E86" s="9"/>
+      <c r="F86" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G86" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="H86" s="40"/>
-      <c r="I86" s="41" t="s">
+      <c r="I86" s="8" t="s">
         <v>143</v>
       </c>
     </row>
@@ -3489,20 +3485,19 @@
       <c r="A87" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="B87" s="41" t="s">
+      <c r="B87" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="C87" s="39" t="s">
+      <c r="C87" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D87" s="39"/>
-      <c r="E87" s="39"/>
-      <c r="F87" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G87" s="39"/>
-      <c r="H87" s="40"/>
-      <c r="I87" s="41" t="s">
+      <c r="D87" s="9"/>
+      <c r="E87" s="9"/>
+      <c r="F87" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G87" s="9"/>
+      <c r="I87" s="8" t="s">
         <v>145</v>
       </c>
     </row>
@@ -3510,20 +3505,19 @@
       <c r="A88" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="B88" s="41" t="s">
+      <c r="B88" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="C88" s="39" t="s">
+      <c r="C88" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D88" s="39"/>
-      <c r="E88" s="39"/>
-      <c r="F88" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G88" s="39"/>
-      <c r="H88" s="40"/>
-      <c r="I88" s="41" t="s">
+      <c r="D88" s="9"/>
+      <c r="E88" s="9"/>
+      <c r="F88" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G88" s="9"/>
+      <c r="I88" s="8" t="s">
         <v>147</v>
       </c>
     </row>
@@ -3531,18 +3525,17 @@
       <c r="A89" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="B89" s="41" t="s">
+      <c r="B89" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="C89" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D89" s="39"/>
-      <c r="E89" s="39"/>
-      <c r="F89" s="39"/>
-      <c r="G89" s="39"/>
-      <c r="H89" s="40"/>
-      <c r="I89" s="41" t="s">
+      <c r="C89" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D89" s="9"/>
+      <c r="E89" s="9"/>
+      <c r="F89" s="9"/>
+      <c r="G89" s="9"/>
+      <c r="I89" s="8" t="s">
         <v>149</v>
       </c>
     </row>
@@ -3550,24 +3543,24 @@
       <c r="A90" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="B90" s="41" t="s">
+      <c r="B90" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="C90" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D90" s="39"/>
-      <c r="E90" s="39" t="s">
+      <c r="C90" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D90" s="9"/>
+      <c r="E90" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F90" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G90" s="39"/>
-      <c r="H90" s="40" t="s">
+      <c r="F90" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G90" s="9"/>
+      <c r="H90" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="I90" s="41" t="s">
+      <c r="I90" s="8" t="s">
         <v>152</v>
       </c>
     </row>
@@ -3575,24 +3568,24 @@
       <c r="A91" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="B91" s="41" t="s">
+      <c r="B91" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="C91" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D91" s="39"/>
-      <c r="E91" s="39" t="s">
+      <c r="C91" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D91" s="9"/>
+      <c r="E91" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F91" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G91" s="39"/>
-      <c r="H91" s="40" t="s">
+      <c r="F91" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G91" s="9"/>
+      <c r="H91" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="I91" s="41" t="s">
+      <c r="I91" s="8" t="s">
         <v>154</v>
       </c>
     </row>
@@ -3600,735 +3593,887 @@
       <c r="A92" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="B92" s="41" t="s">
+      <c r="B92" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="C92" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D92" s="39"/>
-      <c r="E92" s="39" t="s">
+      <c r="C92" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D92" s="9"/>
+      <c r="E92" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F92" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G92" s="39"/>
-      <c r="H92" s="40" t="s">
+      <c r="F92" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G92" s="9"/>
+      <c r="H92" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="I92" s="41" t="s">
+      <c r="I92" s="8" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="42" t="s">
+      <c r="A93" s="39" t="s">
         <v>157</v>
       </c>
-      <c r="B93" s="41" t="s">
+      <c r="B93" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C93" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D93" s="39"/>
-      <c r="E93" s="39" t="s">
+      <c r="C93" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D93" s="9"/>
+      <c r="E93" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F93" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G93" s="39" t="s">
+      <c r="F93" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G93" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H93" s="40"/>
-      <c r="I93" s="41" t="s">
+      <c r="I93" s="8" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="42" t="s">
+      <c r="A94" s="39" t="s">
         <v>157</v>
       </c>
-      <c r="B94" s="41" t="s">
+      <c r="B94" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="C94" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D94" s="39"/>
-      <c r="E94" s="39" t="s">
+      <c r="C94" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D94" s="9"/>
+      <c r="E94" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F94" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G94" s="39"/>
-      <c r="H94" s="40" t="s">
+      <c r="F94" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G94" s="9"/>
+      <c r="H94" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="I94" s="41" t="s">
+      <c r="I94" s="8" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="42" t="s">
+      <c r="A95" s="39" t="s">
         <v>157</v>
       </c>
-      <c r="B95" s="41" t="s">
+      <c r="B95" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="C95" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D95" s="39"/>
-      <c r="E95" s="39" t="s">
+      <c r="C95" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D95" s="9"/>
+      <c r="E95" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F95" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G95" s="39" t="s">
+      <c r="F95" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G95" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="H95" s="40" t="s">
+      <c r="H95" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="I95" s="41" t="s">
+      <c r="I95" s="8" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="42" t="s">
+      <c r="A96" s="39" t="s">
         <v>157</v>
       </c>
-      <c r="B96" s="41" t="s">
+      <c r="B96" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="C96" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D96" s="39"/>
-      <c r="E96" s="39" t="s">
+      <c r="C96" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D96" s="9"/>
+      <c r="E96" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F96" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G96" s="39"/>
-      <c r="H96" s="40" t="s">
+      <c r="F96" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G96" s="9"/>
+      <c r="H96" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="I96" s="41" t="s">
+      <c r="I96" s="8" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="42" t="s">
+      <c r="A97" s="39" t="s">
         <v>157</v>
       </c>
-      <c r="B97" s="41" t="s">
+      <c r="B97" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="C97" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D97" s="39"/>
-      <c r="E97" s="39" t="s">
+      <c r="C97" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D97" s="9"/>
+      <c r="E97" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F97" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G97" s="39"/>
-      <c r="H97" s="40" t="s">
+      <c r="F97" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G97" s="9"/>
+      <c r="H97" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="I97" s="41" t="s">
+      <c r="I97" s="8" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="42" t="s">
+      <c r="A98" s="39" t="s">
         <v>157</v>
       </c>
-      <c r="B98" s="41" t="s">
+      <c r="B98" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="C98" s="39" t="s">
+      <c r="C98" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D98" s="39"/>
-      <c r="E98" s="39"/>
-      <c r="F98" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G98" s="39" t="s">
+      <c r="D98" s="9"/>
+      <c r="E98" s="9"/>
+      <c r="F98" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G98" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="H98" s="40"/>
-      <c r="I98" s="41" t="s">
+      <c r="I98" s="8" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="43" t="s">
+      <c r="A99" s="40" t="s">
         <v>168</v>
       </c>
-      <c r="B99" s="41" t="s">
+      <c r="B99" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C99" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D99" s="39"/>
-      <c r="E99" s="39" t="s">
+      <c r="C99" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D99" s="9"/>
+      <c r="E99" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F99" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G99" s="39" t="s">
+      <c r="F99" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G99" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H99" s="40"/>
-      <c r="I99" s="41" t="s">
+      <c r="I99" s="8" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="43" t="s">
+      <c r="A100" s="40" t="s">
         <v>168</v>
       </c>
-      <c r="B100" s="41" t="s">
+      <c r="B100" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="C100" s="39" t="s">
+      <c r="C100" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D100" s="39"/>
-      <c r="E100" s="39"/>
-      <c r="F100" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G100" s="39"/>
-      <c r="H100" s="40"/>
-      <c r="I100" s="41" t="s">
+      <c r="D100" s="9"/>
+      <c r="E100" s="9"/>
+      <c r="F100" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G100" s="9"/>
+      <c r="I100" s="8" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="43" t="s">
+      <c r="A101" s="40" t="s">
         <v>168</v>
       </c>
-      <c r="B101" s="41" t="s">
+      <c r="B101" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C101" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D101" s="39"/>
-      <c r="E101" s="39" t="s">
+      <c r="C101" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D101" s="9"/>
+      <c r="E101" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F101" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G101" s="39"/>
-      <c r="H101" s="40" t="s">
+      <c r="F101" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G101" s="9"/>
+      <c r="H101" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="I101" s="41" t="s">
+      <c r="I101" s="8" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="43" t="s">
+      <c r="A102" s="40" t="s">
         <v>168</v>
       </c>
-      <c r="B102" s="41" t="s">
+      <c r="B102" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C102" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D102" s="39"/>
-      <c r="E102" s="39" t="s">
+      <c r="C102" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D102" s="9"/>
+      <c r="E102" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F102" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G102" s="39"/>
-      <c r="H102" s="40" t="s">
+      <c r="F102" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G102" s="9"/>
+      <c r="H102" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="I102" s="41" t="s">
+      <c r="I102" s="8" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="43" t="s">
+      <c r="A103" s="40" t="s">
         <v>168</v>
       </c>
-      <c r="B103" s="41" t="s">
+      <c r="B103" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C103" s="39" t="s">
+      <c r="C103" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D103" s="39"/>
-      <c r="E103" s="39"/>
-      <c r="F103" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G103" s="39" t="s">
+      <c r="D103" s="9"/>
+      <c r="E103" s="9"/>
+      <c r="F103" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G103" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="H103" s="40"/>
-      <c r="I103" s="41" t="s">
+      <c r="I103" s="8" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="43" t="s">
+      <c r="A104" s="40" t="s">
         <v>168</v>
       </c>
-      <c r="B104" s="41" t="s">
+      <c r="B104" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C104" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D104" s="39"/>
-      <c r="E104" s="39"/>
-      <c r="F104" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G104" s="39" t="s">
+      <c r="C104" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D104" s="9"/>
+      <c r="E104" s="9"/>
+      <c r="F104" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G104" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="H104" s="40"/>
-      <c r="I104" s="41" t="s">
+      <c r="I104" s="8" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="44" t="s">
+      <c r="A105" s="41" t="s">
         <v>176</v>
       </c>
-      <c r="B105" s="41" t="s">
+      <c r="B105" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C105" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D105" s="39"/>
-      <c r="E105" s="39" t="s">
+      <c r="C105" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D105" s="9"/>
+      <c r="E105" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F105" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G105" s="39" t="s">
+      <c r="F105" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G105" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H105" s="40"/>
-      <c r="I105" s="41" t="s">
+      <c r="I105" s="8" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="44" t="s">
+      <c r="A106" s="41" t="s">
         <v>176</v>
       </c>
-      <c r="B106" s="41" t="s">
+      <c r="B106" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C106" s="39" t="s">
+      <c r="C106" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D106" s="39"/>
-      <c r="E106" s="39"/>
-      <c r="F106" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G106" s="39"/>
-      <c r="H106" s="40"/>
-      <c r="I106" s="41" t="s">
+      <c r="D106" s="9"/>
+      <c r="E106" s="9"/>
+      <c r="F106" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G106" s="9"/>
+      <c r="I106" s="8" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="44" t="s">
+      <c r="A107" s="41" t="s">
         <v>176</v>
       </c>
-      <c r="B107" s="41" t="s">
+      <c r="B107" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C107" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D107" s="39"/>
-      <c r="E107" s="39"/>
-      <c r="F107" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G107" s="39" t="s">
+      <c r="C107" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D107" s="9"/>
+      <c r="E107" s="9"/>
+      <c r="F107" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G107" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="H107" s="40"/>
-      <c r="I107" s="41" t="s">
+      <c r="I107" s="8" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="45" t="s">
+      <c r="A108" s="42" t="s">
         <v>180</v>
       </c>
-      <c r="B108" s="41" t="s">
+      <c r="B108" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="C108" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D108" s="39"/>
-      <c r="E108" s="39" t="s">
+      <c r="C108" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D108" s="9"/>
+      <c r="E108" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F108" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G108" s="39"/>
-      <c r="H108" s="40" t="s">
+      <c r="F108" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G108" s="9"/>
+      <c r="H108" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="I108" s="41" t="s">
+      <c r="I108" s="8" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="45" t="s">
+      <c r="A109" s="42" t="s">
         <v>180</v>
       </c>
-      <c r="B109" s="41" t="s">
+      <c r="B109" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="C109" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D109" s="39"/>
-      <c r="E109" s="39" t="s">
+      <c r="C109" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D109" s="9"/>
+      <c r="E109" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F109" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G109" s="39" t="s">
+      <c r="F109" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G109" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="H109" s="40" t="s">
+      <c r="H109" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="I109" s="41" t="s">
+      <c r="I109" s="8" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="45" t="s">
+      <c r="A110" s="42" t="s">
         <v>180</v>
       </c>
-      <c r="B110" s="41" t="s">
+      <c r="B110" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="C110" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D110" s="39"/>
-      <c r="E110" s="39"/>
-      <c r="F110" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G110" s="39"/>
-      <c r="H110" s="40"/>
-      <c r="I110" s="41" t="s">
+      <c r="C110" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D110" s="9"/>
+      <c r="E110" s="9"/>
+      <c r="F110" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G110" s="9"/>
+      <c r="I110" s="8" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="45" t="s">
+      <c r="A111" s="42" t="s">
         <v>180</v>
       </c>
-      <c r="B111" s="41" t="s">
+      <c r="B111" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="C111" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D111" s="39"/>
-      <c r="E111" s="39"/>
-      <c r="F111" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G111" s="39"/>
-      <c r="H111" s="40"/>
-      <c r="I111" s="41" t="s">
+      <c r="C111" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D111" s="9"/>
+      <c r="E111" s="9"/>
+      <c r="F111" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G111" s="9"/>
+      <c r="I111" s="8" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="45" t="s">
+      <c r="A112" s="42" t="s">
         <v>180</v>
       </c>
-      <c r="B112" s="41" t="s">
+      <c r="B112" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="C112" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D112" s="39"/>
-      <c r="E112" s="39" t="s">
+      <c r="C112" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D112" s="9"/>
+      <c r="E112" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F112" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G112" s="39"/>
-      <c r="H112" s="40" t="s">
+      <c r="F112" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G112" s="9"/>
+      <c r="H112" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="I112" s="41" t="s">
+      <c r="I112" s="8" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="45" t="s">
+      <c r="A113" s="42" t="s">
         <v>180</v>
       </c>
-      <c r="B113" s="41" t="s">
+      <c r="B113" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="C113" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D113" s="39"/>
-      <c r="E113" s="39" t="s">
+      <c r="C113" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D113" s="9"/>
+      <c r="E113" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F113" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G113" s="39"/>
-      <c r="H113" s="40" t="s">
+      <c r="F113" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G113" s="9"/>
+      <c r="H113" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="I113" s="41" t="s">
+      <c r="I113" s="8" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="45" t="s">
+      <c r="A114" s="42" t="s">
         <v>180</v>
       </c>
-      <c r="B114" s="41" t="s">
+      <c r="B114" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="C114" s="39" t="s">
+      <c r="C114" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D114" s="39"/>
-      <c r="E114" s="39"/>
-      <c r="F114" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G114" s="39" t="s">
+      <c r="D114" s="9"/>
+      <c r="E114" s="9"/>
+      <c r="F114" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G114" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="H114" s="40"/>
-      <c r="I114" s="41" t="s">
+      <c r="I114" s="8" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="46" t="s">
+      <c r="A115" s="43" t="s">
         <v>191</v>
       </c>
-      <c r="B115" s="41" t="s">
+      <c r="B115" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C115" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D115" s="39"/>
-      <c r="E115" s="39" t="s">
+      <c r="C115" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D115" s="9"/>
+      <c r="E115" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F115" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G115" s="39" t="s">
+      <c r="F115" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G115" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H115" s="40"/>
-      <c r="I115" s="41" t="s">
+      <c r="I115" s="8" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="46" t="s">
+      <c r="A116" s="43" t="s">
         <v>191</v>
       </c>
-      <c r="B116" s="41" t="s">
+      <c r="B116" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="C116" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D116" s="39"/>
-      <c r="E116" s="39" t="s">
+      <c r="C116" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D116" s="9"/>
+      <c r="E116" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F116" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G116" s="39"/>
-      <c r="H116" s="40" t="s">
+      <c r="F116" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G116" s="9"/>
+      <c r="H116" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="I116" s="41" t="s">
+      <c r="I116" s="8" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="46" t="s">
+      <c r="A117" s="43" t="s">
         <v>191</v>
       </c>
-      <c r="B117" s="41" t="s">
+      <c r="B117" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="C117" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D117" s="39"/>
-      <c r="E117" s="39" t="s">
+      <c r="C117" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D117" s="9"/>
+      <c r="E117" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F117" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G117" s="39"/>
-      <c r="H117" s="40" t="s">
+      <c r="F117" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G117" s="9"/>
+      <c r="H117" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="I117" s="41" t="s">
+      <c r="I117" s="8" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="46" t="s">
+      <c r="A118" s="43" t="s">
         <v>191</v>
       </c>
-      <c r="B118" s="41" t="s">
+      <c r="B118" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="C118" s="39" t="s">
+      <c r="C118" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D118" s="39"/>
-      <c r="E118" s="39"/>
-      <c r="F118" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G118" s="39" t="s">
+      <c r="D118" s="9"/>
+      <c r="E118" s="9"/>
+      <c r="F118" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G118" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="H118" s="40"/>
-      <c r="I118" s="41" t="s">
+      <c r="I118" s="8" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="46" t="s">
+      <c r="A119" s="43" t="s">
         <v>191</v>
       </c>
-      <c r="B119" s="41" t="s">
+      <c r="B119" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="C119" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D119" s="39"/>
-      <c r="E119" s="39"/>
-      <c r="F119" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G119" s="39"/>
-      <c r="H119" s="40"/>
-      <c r="I119" s="41" t="s">
+      <c r="C119" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D119" s="9"/>
+      <c r="E119" s="9"/>
+      <c r="F119" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G119" s="9"/>
+      <c r="I119" s="8" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="46" t="s">
+      <c r="A120" s="43" t="s">
         <v>191</v>
       </c>
-      <c r="B120" s="41" t="s">
+      <c r="B120" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="C120" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D120" s="39"/>
-      <c r="E120" s="39" t="s">
+      <c r="C120" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D120" s="9"/>
+      <c r="E120" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F120" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G120" s="39"/>
-      <c r="H120" s="40" t="s">
+      <c r="F120" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G120" s="9"/>
+      <c r="H120" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="I120" s="41" t="s">
+      <c r="I120" s="8" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="46" t="s">
+      <c r="A121" s="43" t="s">
         <v>191</v>
       </c>
-      <c r="B121" s="41" t="s">
+      <c r="B121" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="C121" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D121" s="39"/>
-      <c r="E121" s="39" t="s">
+      <c r="C121" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D121" s="9"/>
+      <c r="E121" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F121" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="G121" s="39"/>
-      <c r="H121" s="40" t="s">
+      <c r="F121" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G121" s="9"/>
+      <c r="H121" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="I121" s="41" t="s">
+      <c r="I121" s="8" t="s">
         <v>156</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="B122" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C122" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D122" s="14"/>
+      <c r="E122" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F122" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G122" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="H122" s="15"/>
+      <c r="I122" s="16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C123" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D123" s="14"/>
+      <c r="E123" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F123" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G123" s="13"/>
+      <c r="H123" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="I123" s="16" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C124" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D124" s="14"/>
+      <c r="E124" s="14"/>
+      <c r="F124" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G124" s="13"/>
+      <c r="H124" s="15"/>
+      <c r="I124" s="16" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C125" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D125" s="14"/>
+      <c r="E125" s="14"/>
+      <c r="F125" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G125" s="13"/>
+      <c r="H125" s="15"/>
+      <c r="I125" s="16" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C126" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D126" s="14"/>
+      <c r="E126" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F126" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G126" s="13"/>
+      <c r="H126" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="I126" s="45" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="B127" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C127" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D127" s="14"/>
+      <c r="E127" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F127" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G127" s="13"/>
+      <c r="H127" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="I127" s="16" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C128" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D128" s="14"/>
+      <c r="E128" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="F128" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G128" s="46" t="s">
+        <v>140</v>
+      </c>
+      <c r="H128" s="15"/>
+      <c r="I128" s="45" t="s">
+        <v>209</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C15:C26 C28:C31 C33:C54" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C15:C26 C28:C31 C33:C54 C122:C128" type="list">
       <formula1>Validações!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E15:E26 E28:E31 E33:E54" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E15:E26 E28:E31 E33:E54 E122:E128" type="list">
       <formula1>Validações!$B$1:$B$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F15:F26 F28:F31 F33:F54" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F15:F26 F28:F31 F33:F54 F122:F128" type="list">
       <formula1>Validações!$C$1:$C$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4363,361 +4508,361 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="47" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B4" s="48" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="47" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="B5" s="48" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="47" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="B6" s="48" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="47" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="B7" s="48" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="47" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="B8" s="48" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="47" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="B9" s="48" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="47" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="B10" s="48" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="47" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="B11" s="48" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="47" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="B12" s="48" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="49" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="50" t="s">
+      <c r="A16" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="50" t="s">
-        <v>223</v>
-      </c>
-      <c r="C16" s="50" t="s">
+      <c r="B16" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D16" s="50" t="s">
+      <c r="D16" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="50" t="s">
+      <c r="E16" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F16" s="50" t="s">
+      <c r="F16" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G16" s="50" t="s">
-        <v>224</v>
-      </c>
-      <c r="H16" s="50" t="s">
-        <v>225</v>
-      </c>
-      <c r="I16" s="50" t="s">
+      <c r="G16" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="I16" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="51" t="s">
-        <v>226</v>
-      </c>
-      <c r="B17" s="51" t="s">
-        <v>227</v>
-      </c>
-      <c r="C17" s="52" t="s">
+      <c r="A17" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="C17" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="D17" s="53" t="s">
-        <v>228</v>
-      </c>
-      <c r="E17" s="53" t="s">
+      <c r="D17" s="14" t="s">
+        <v>236</v>
+      </c>
+      <c r="E17" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="F17" s="53" t="s">
-        <v>21</v>
-      </c>
-      <c r="G17" s="52" t="s">
-        <v>229</v>
-      </c>
-      <c r="H17" s="51" t="s">
-        <v>230</v>
-      </c>
-      <c r="I17" s="54" t="s">
-        <v>231</v>
+      <c r="F17" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="I17" s="16" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="55" t="s">
-        <v>226</v>
-      </c>
-      <c r="B18" s="55" t="s">
-        <v>232</v>
-      </c>
-      <c r="C18" s="56" t="s">
-        <v>233</v>
-      </c>
-      <c r="D18" s="57" t="s">
+      <c r="A18" s="15" t="s">
         <v>234</v>
       </c>
-      <c r="E18" s="57" t="s">
+      <c r="B18" s="15" t="s">
+        <v>240</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>242</v>
+      </c>
+      <c r="E18" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="F18" s="57" t="s">
-        <v>21</v>
-      </c>
-      <c r="G18" s="56" t="s">
-        <v>230</v>
-      </c>
-      <c r="H18" s="55" t="s">
-        <v>235</v>
+      <c r="F18" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="H18" s="15" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="51" t="s">
-        <v>226</v>
-      </c>
-      <c r="B19" s="51" t="s">
+      <c r="A19" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>241</v>
+      </c>
+      <c r="D19" s="14" t="s">
         <v>236</v>
       </c>
-      <c r="C19" s="52" t="s">
-        <v>233</v>
-      </c>
-      <c r="D19" s="53" t="s">
-        <v>228</v>
-      </c>
-      <c r="E19" s="53" t="s">
+      <c r="E19" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="F19" s="53" t="s">
-        <v>21</v>
-      </c>
-      <c r="G19" s="52" t="s">
-        <v>230</v>
-      </c>
-      <c r="H19" s="51" t="s">
+      <c r="F19" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G19" s="13" t="s">
+        <v>238</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="15" t="s">
+        <v>234</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>246</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>238</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="H20" s="15" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>241</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="G21" s="13" t="s">
+        <v>249</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="15" t="s">
+        <v>234</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>251</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="H22" s="15" t="s">
+        <v>252</v>
+      </c>
+      <c r="I22" s="19" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
+        <v>254</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>236</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" s="13" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="55" t="s">
-        <v>226</v>
-      </c>
-      <c r="B20" s="55" t="s">
+      <c r="H23" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="C20" s="56" t="s">
-        <v>239</v>
-      </c>
-      <c r="D20" s="57" t="s">
-        <v>230</v>
-      </c>
-      <c r="E20" s="57" t="s">
+      <c r="I23" s="16" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="15" t="s">
+        <v>254</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>256</v>
+      </c>
+      <c r="C24" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>257</v>
+      </c>
+      <c r="E24" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="F20" s="57" t="s">
-        <v>21</v>
-      </c>
-      <c r="G20" s="56" t="s">
-        <v>230</v>
-      </c>
-      <c r="H20" s="55" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="51" t="s">
-        <v>226</v>
-      </c>
-      <c r="B21" s="51" t="s">
-        <v>67</v>
-      </c>
-      <c r="C21" s="52" t="s">
-        <v>233</v>
-      </c>
-      <c r="D21" s="53" t="s">
-        <v>234</v>
-      </c>
-      <c r="E21" s="53" t="s">
+      <c r="F24" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="H24" s="15" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
+        <v>254</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>259</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="E25" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="F21" s="53" t="s">
-        <v>63</v>
-      </c>
-      <c r="G21" s="52" t="s">
-        <v>241</v>
-      </c>
-      <c r="H21" s="51" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="55" t="s">
-        <v>226</v>
-      </c>
-      <c r="B22" s="55" t="s">
-        <v>243</v>
-      </c>
-      <c r="C22" s="56" t="s">
-        <v>39</v>
-      </c>
-      <c r="D22" s="57" t="s">
-        <v>228</v>
-      </c>
-      <c r="E22" s="57" t="s">
-        <v>28</v>
-      </c>
-      <c r="F22" s="57" t="s">
-        <v>21</v>
-      </c>
-      <c r="G22" s="56" t="s">
-        <v>230</v>
-      </c>
-      <c r="H22" s="55" t="s">
-        <v>244</v>
-      </c>
-      <c r="I22" s="58" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="51" t="s">
-        <v>246</v>
-      </c>
-      <c r="B23" s="51" t="s">
-        <v>243</v>
-      </c>
-      <c r="C23" s="52" t="s">
-        <v>39</v>
-      </c>
-      <c r="D23" s="53" t="s">
-        <v>228</v>
-      </c>
-      <c r="E23" s="53" t="s">
-        <v>20</v>
-      </c>
-      <c r="F23" s="53" t="s">
-        <v>21</v>
-      </c>
-      <c r="G23" s="52" t="s">
-        <v>229</v>
-      </c>
-      <c r="H23" s="51" t="s">
-        <v>230</v>
-      </c>
-      <c r="I23" s="54" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="55" t="s">
-        <v>246</v>
-      </c>
-      <c r="B24" s="55" t="s">
-        <v>248</v>
-      </c>
-      <c r="C24" s="56" t="s">
-        <v>233</v>
-      </c>
-      <c r="D24" s="57" t="s">
-        <v>249</v>
-      </c>
-      <c r="E24" s="57" t="s">
-        <v>42</v>
-      </c>
-      <c r="F24" s="57" t="s">
-        <v>21</v>
-      </c>
-      <c r="G24" s="56" t="s">
-        <v>230</v>
-      </c>
-      <c r="H24" s="55" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="51" t="s">
-        <v>246</v>
-      </c>
-      <c r="B25" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="C25" s="52" t="s">
-        <v>39</v>
-      </c>
-      <c r="D25" s="53" t="s">
-        <v>252</v>
-      </c>
-      <c r="E25" s="53" t="s">
-        <v>42</v>
-      </c>
-      <c r="F25" s="53" t="s">
-        <v>21</v>
-      </c>
-      <c r="G25" s="52" t="s">
-        <v>253</v>
-      </c>
-      <c r="H25" s="51" t="s">
-        <v>254</v>
+      <c r="F25" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -4752,7 +4897,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>28</v>
@@ -4763,15 +4908,15 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>42</v>
@@ -4779,7 +4924,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4789,27 +4934,27 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
atualização do dicionario e criação das triggers de adicionar e deletar e verificar estoque
</commit_message>
<xml_diff>
--- a/documentos/modelo_dicionario_de_dados.xlsx
+++ b/documentos/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="888" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="961" uniqueCount="284">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -652,6 +652,42 @@
   </si>
   <si>
     <t xml:space="preserve">Data e hora da compra da peça.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">saida_peca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primaria de identificação da saida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quantidade_saida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantidade que foi baixada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valor_saida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor da compra </t>
+  </si>
+  <si>
+    <t xml:space="preserve">numero_serie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Número de série</t>
+  </si>
+  <si>
+    <t xml:space="preserve">numero_lote</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Número de lote</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHECK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_saida</t>
   </si>
   <si>
     <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
@@ -943,9 +979,8 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <family val="0"/>
     </font>
     <font>
       <b val="true"/>
@@ -956,7 +991,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="24">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1002,7 +1037,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF6D"/>
-        <bgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF38"/>
       </patternFill>
     </fill>
     <fill>
@@ -1083,6 +1118,18 @@
         <bgColor rgb="FF4C78A8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF38"/>
+        <bgColor rgb="FFFFFF6D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
@@ -1133,7 +1180,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="52">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1310,7 +1357,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1318,8 +1373,8 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="23" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -1350,7 +1405,7 @@
       <rgbColor rgb="FFFF3838"/>
       <rgbColor rgb="FF00FF7F"/>
       <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFFFF38"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF990000"/>
@@ -1586,7 +1641,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J128"/>
+  <dimension ref="A1:J140"/>
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
@@ -4300,7 +4355,7 @@
       <c r="A122" s="44" t="s">
         <v>202</v>
       </c>
-      <c r="B122" s="0" t="s">
+      <c r="B122" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C122" s="13" t="s">
@@ -4409,11 +4464,11 @@
       <c r="H126" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="I126" s="45" t="s">
+      <c r="I126" s="22" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="44" t="s">
         <v>202</v>
       </c>
@@ -4455,25 +4510,301 @@
       <c r="F128" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G128" s="46" t="s">
+      <c r="G128" s="45" t="s">
         <v>140</v>
       </c>
       <c r="H128" s="15"/>
-      <c r="I128" s="45" t="s">
+      <c r="I128" s="22" t="s">
         <v>209</v>
       </c>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C129" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D129" s="14"/>
+      <c r="E129" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F129" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G129" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="H129" s="15"/>
+      <c r="I129" s="47" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C130" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D130" s="14"/>
+      <c r="E130" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F130" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G130" s="13"/>
+      <c r="H130" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="I130" s="16" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C131" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D131" s="14"/>
+      <c r="E131" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F131" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="G131" s="13"/>
+      <c r="H131" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I131" s="16" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C132" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D132" s="14"/>
+      <c r="E132" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F132" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G132" s="13"/>
+      <c r="H132" s="15"/>
+      <c r="I132" s="16" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C133" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D133" s="14"/>
+      <c r="E133" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F133" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G133" s="13"/>
+      <c r="H133" s="15"/>
+      <c r="I133" s="16" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C134" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D134" s="14"/>
+      <c r="E134" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F134" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G134" s="13"/>
+      <c r="H134" s="15"/>
+      <c r="I134" s="16" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="C135" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D135" s="14"/>
+      <c r="E135" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F135" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G135" s="13"/>
+      <c r="H135" s="15"/>
+      <c r="I135" s="16" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="B136" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="C136" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D136" s="9"/>
+      <c r="E136" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F136" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G136" s="9"/>
+      <c r="H136" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I136" s="8" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="B137" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="C137" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D137" s="9"/>
+      <c r="E137" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F137" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G137" s="9"/>
+      <c r="H137" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="I137" s="8" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="B138" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C138" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D138" s="14"/>
+      <c r="E138" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F138" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G138" s="13" t="s">
+        <v>220</v>
+      </c>
+      <c r="H138" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="I138" s="16" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="46" t="s">
+        <v>210</v>
+      </c>
+      <c r="B139" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="C139" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D139" s="9"/>
+      <c r="E139" s="9"/>
+      <c r="F139" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G139" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="I139" s="8" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="48"/>
+      <c r="C140" s="13"/>
+      <c r="D140" s="14"/>
+      <c r="E140" s="14"/>
+      <c r="F140" s="14"/>
+      <c r="G140" s="13"/>
+      <c r="H140" s="15"/>
+      <c r="I140" s="16"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C15:C26 C28:C31 C33:C54 C122:C128" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C15:C26 C28:C31 C33:C54 C122:C135 C138 C140" type="list">
       <formula1>Validações!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E15:E26 E28:E31 E33:E54 E122:E128" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E15:E26 E28:E31 E33:E54 E122:E135 E138 E140" type="list">
       <formula1>Validações!$B$1:$B$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F15:F26 F28:F31 F33:F54 F122:F128" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F15:F26 F28:F31 F33:F54 F122:F135 F138 F140" type="list">
       <formula1>Validações!$C$1:$C$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4508,89 +4839,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="47" t="s">
-        <v>212</v>
-      </c>
-      <c r="B4" s="48" t="s">
-        <v>213</v>
+      <c r="A4" s="49" t="s">
+        <v>224</v>
+      </c>
+      <c r="B4" s="50" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="47" t="s">
-        <v>214</v>
-      </c>
-      <c r="B5" s="48" t="s">
-        <v>215</v>
+      <c r="A5" s="49" t="s">
+        <v>226</v>
+      </c>
+      <c r="B5" s="50" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="47" t="s">
-        <v>216</v>
-      </c>
-      <c r="B6" s="48" t="s">
-        <v>217</v>
+      <c r="A6" s="49" t="s">
+        <v>228</v>
+      </c>
+      <c r="B6" s="50" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="47" t="s">
-        <v>218</v>
-      </c>
-      <c r="B7" s="48" t="s">
-        <v>219</v>
+      <c r="A7" s="49" t="s">
+        <v>230</v>
+      </c>
+      <c r="B7" s="50" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="47" t="s">
-        <v>220</v>
-      </c>
-      <c r="B8" s="48" t="s">
-        <v>221</v>
+      <c r="A8" s="49" t="s">
+        <v>232</v>
+      </c>
+      <c r="B8" s="50" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="47" t="s">
-        <v>222</v>
-      </c>
-      <c r="B9" s="48" t="s">
-        <v>223</v>
+      <c r="A9" s="49" t="s">
+        <v>234</v>
+      </c>
+      <c r="B9" s="50" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="47" t="s">
-        <v>224</v>
-      </c>
-      <c r="B10" s="48" t="s">
-        <v>225</v>
+      <c r="A10" s="49" t="s">
+        <v>236</v>
+      </c>
+      <c r="B10" s="50" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="47" t="s">
-        <v>226</v>
-      </c>
-      <c r="B11" s="48" t="s">
-        <v>227</v>
+      <c r="A11" s="49" t="s">
+        <v>238</v>
+      </c>
+      <c r="B11" s="50" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="47" t="s">
-        <v>228</v>
-      </c>
-      <c r="B12" s="48" t="s">
-        <v>229</v>
+      <c r="A12" s="49" t="s">
+        <v>240</v>
+      </c>
+      <c r="B12" s="50" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="49" t="s">
-        <v>230</v>
+      <c r="A14" s="51" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4598,7 +4929,7 @@
         <v>8</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>10</v>
@@ -4613,10 +4944,10 @@
         <v>13</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="I16" s="6" t="s">
         <v>16</v>
@@ -4624,16 +4955,16 @@
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>39</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="E17" s="14" t="s">
         <v>20</v>
@@ -4642,27 +4973,27 @@
         <v>21</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="I17" s="16" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="15" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="E18" s="18" t="s">
         <v>42</v>
@@ -4671,24 +5002,24 @@
         <v>21</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="E19" s="14" t="s">
         <v>42</v>
@@ -4697,24 +5028,24 @@
         <v>21</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="E20" s="18" t="s">
         <v>42</v>
@@ -4723,24 +5054,24 @@
         <v>21</v>
       </c>
       <c r="G20" s="17" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>67</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="E21" s="14" t="s">
         <v>42</v>
@@ -4749,24 +5080,24 @@
         <v>63</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="C22" s="17" t="s">
         <v>39</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="E22" s="18" t="s">
         <v>28</v>
@@ -4775,27 +5106,27 @@
         <v>21</v>
       </c>
       <c r="G22" s="17" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="H22" s="15" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="I22" s="19" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>39</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>20</v>
@@ -4804,27 +5135,27 @@
         <v>21</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="I23" s="16" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="E24" s="18" t="s">
         <v>42</v>
@@ -4833,24 +5164,24 @@
         <v>21</v>
       </c>
       <c r="G24" s="17" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="H24" s="15" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>39</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="E25" s="14" t="s">
         <v>42</v>
@@ -4859,10 +5190,10 @@
         <v>21</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -4897,7 +5228,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>28</v>
@@ -4908,15 +5239,15 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>42</v>
@@ -4924,7 +5255,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4934,27 +5265,27 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>268</v>
+        <v>280</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>